<commit_message>
Features: Adicionados relatórios Mensais e Anuais. Bem como ajustes no semanal
</commit_message>
<xml_diff>
--- a/calendarioDinamico/backend/reports/report-69b9afeb326f8b16987ab4a9.xlsx
+++ b/calendarioDinamico/backend/reports/report-69b9afeb326f8b16987ab4a9.xlsx
@@ -11,12 +11,33 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Dia</t>
   </si>
   <si>
     <t>Pontos</t>
+  </si>
+  <si>
+    <t>Segunda</t>
+  </si>
+  <si>
+    <t>Terça</t>
+  </si>
+  <si>
+    <t>Quarta</t>
+  </si>
+  <si>
+    <t>Quinta</t>
+  </si>
+  <si>
+    <t>Sexta</t>
+  </si>
+  <si>
+    <t>Sábado</t>
+  </si>
+  <si>
+    <t>Domingo</t>
   </si>
   <si>
     <t>TOTAL</t>
@@ -396,7 +417,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -411,11 +432,67 @@
         <v>1</v>
       </c>
     </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+    </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10">
         <v>0</v>
       </c>
     </row>

</xml_diff>